<commit_message>
Cierre 2026-10-20 16:11 — Revision TOTAL CODE
</commit_message>
<xml_diff>
--- a/Presupuestos/Obras/Obra005/Precios/TorcuatoMateriales.xlsx
+++ b/Presupuestos/Obras/Obra005/Precios/TorcuatoMateriales.xlsx
@@ -791,11 +791,11 @@
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>m2</t>
+          <t>Kg</t>
         </is>
       </c>
       <c r="D19" t="n">
-        <v>20000</v>
+        <v>800</v>
       </c>
     </row>
     <row r="20">

</xml_diff>